<commit_message>
Merge BookYourData contacts into marina prospect list
Adds 49 purchased-list contacts (all with deliverable-flagged emails and
named people) to the researched marina list, deduplicated by email and
by company against the existing rows. Total is now 289 prospects, 178
with email addresses.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HDNuNJyMUYHgzmqi83Vpfz
</commit_message>
<xml_diff>
--- a/orange_peel_marina_prospects.xlsx
+++ b/orange_peel_marina_prospects.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Marina Prospects" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Marina Prospects'!$A$1:$M$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Marina Prospects'!$A$1:$M$290</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M241"/>
+  <dimension ref="A1:M290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -448,7 +448,7 @@
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="36" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -13211,8 +13211,3203 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>Braga</t>
+        </is>
+      </c>
+      <c r="C242" s="2" t="inlineStr">
+        <is>
+          <t>mike@kofloorsupply.com</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>9738515755</t>
+        </is>
+      </c>
+      <c r="E242" s="2" t="inlineStr">
+        <is>
+          <t>Store Manager</t>
+        </is>
+      </c>
+      <c r="F242" s="2" t="inlineStr">
+        <is>
+          <t>Ko Floor Supply</t>
+        </is>
+      </c>
+      <c r="G242" s="2" t="inlineStr">
+        <is>
+          <t>https://kofloorsupply.com</t>
+        </is>
+      </c>
+      <c r="H242" s="2" t="inlineStr">
+        <is>
+          <t>8 North Corporate Drive</t>
+        </is>
+      </c>
+      <c r="I242" s="2" t="inlineStr">
+        <is>
+          <t>Riverdale</t>
+        </is>
+      </c>
+      <c r="J242" s="2" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="K242" s="2" t="inlineStr">
+        <is>
+          <t>07457</t>
+        </is>
+      </c>
+      <c r="L242" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M242" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Nondurable goods, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="B243" s="2" t="inlineStr">
+        <is>
+          <t>Kraus</t>
+        </is>
+      </c>
+      <c r="C243" s="2" t="inlineStr">
+        <is>
+          <t>daniel.kraus@noblehousehotels.com</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>+1 425-827-8737</t>
+        </is>
+      </c>
+      <c r="E243" s="2" t="inlineStr">
+        <is>
+          <t>General Manager   Six Seven Restaurant   Lounge   Edgewater Hotel</t>
+        </is>
+      </c>
+      <c r="F243" s="2" t="inlineStr">
+        <is>
+          <t>Noble House Hotels &amp; Resorts</t>
+        </is>
+      </c>
+      <c r="G243" s="2" t="inlineStr">
+        <is>
+          <t>https://noblehousehotels.com</t>
+        </is>
+      </c>
+      <c r="H243" s="2" t="inlineStr">
+        <is>
+          <t>600 6th Street South</t>
+        </is>
+      </c>
+      <c r="I243" s="2" t="inlineStr">
+        <is>
+          <t>Juanita</t>
+        </is>
+      </c>
+      <c r="J243" s="2" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="K243" s="2" t="inlineStr">
+        <is>
+          <t>98033</t>
+        </is>
+      </c>
+      <c r="L243" s="2" t="inlineStr">
+        <is>
+          <t>Pacific Northwest - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M243" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Hotels and motels</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>Rob</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>Jones</t>
+        </is>
+      </c>
+      <c r="C244" s="2" t="inlineStr">
+        <is>
+          <t>rjones4192@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>+1 800-287-9060</t>
+        </is>
+      </c>
+      <c r="E244" s="2" t="inlineStr">
+        <is>
+          <t>General Sales Manager</t>
+        </is>
+      </c>
+      <c r="F244" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G244" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H244" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I244" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J244" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K244" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L244" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M244" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>Jenole</t>
+        </is>
+      </c>
+      <c r="B245" s="2" t="inlineStr">
+        <is>
+          <t>Peacock</t>
+        </is>
+      </c>
+      <c r="C245" s="2" t="inlineStr">
+        <is>
+          <t>jenolepeacock@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>+13603176192</t>
+        </is>
+      </c>
+      <c r="E245" s="2" t="inlineStr">
+        <is>
+          <t>Cascade Bay Grill Store Manager And Retail Buyer</t>
+        </is>
+      </c>
+      <c r="F245" s="2" t="inlineStr">
+        <is>
+          <t>Rosario Resort &amp; Spa</t>
+        </is>
+      </c>
+      <c r="G245" s="2" t="inlineStr">
+        <is>
+          <t>https://rosarioresort.com</t>
+        </is>
+      </c>
+      <c r="H245" s="2" t="inlineStr">
+        <is>
+          <t>1400 Rosario Road</t>
+        </is>
+      </c>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>Eastsound</t>
+        </is>
+      </c>
+      <c r="J245" s="2" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="K245" s="2" t="inlineStr">
+        <is>
+          <t>98245</t>
+        </is>
+      </c>
+      <c r="L245" s="2" t="inlineStr">
+        <is>
+          <t>Pacific Northwest - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M245" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Hotels and motels</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>Megan</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>Brevak</t>
+        </is>
+      </c>
+      <c r="C246" s="2" t="inlineStr">
+        <is>
+          <t>mbrevak@barkers-island-marina.com</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>+1 715-392-7152</t>
+        </is>
+      </c>
+      <c r="E246" s="2" t="inlineStr">
+        <is>
+          <t>Store Manager And Communication Specialist</t>
+        </is>
+      </c>
+      <c r="F246" s="2" t="inlineStr">
+        <is>
+          <t>Barkers Island Marina</t>
+        </is>
+      </c>
+      <c r="G246" s="2" t="inlineStr">
+        <is>
+          <t>https://barkers-island-marina.com</t>
+        </is>
+      </c>
+      <c r="H246" s="2" t="inlineStr">
+        <is>
+          <t>250 Marina Dr</t>
+        </is>
+      </c>
+      <c r="I246" s="2" t="inlineStr">
+        <is>
+          <t>Oliver</t>
+        </is>
+      </c>
+      <c r="J246" s="2" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="K246" s="2" t="inlineStr">
+        <is>
+          <t>54880</t>
+        </is>
+      </c>
+      <c r="L246" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M246" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Amusement and recreation, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>Kathy</t>
+        </is>
+      </c>
+      <c r="B247" s="2" t="inlineStr">
+        <is>
+          <t>Garcia</t>
+        </is>
+      </c>
+      <c r="C247" s="2" t="inlineStr">
+        <is>
+          <t>kathyg@portofbremerton.org</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>+1 360-674-2381</t>
+        </is>
+      </c>
+      <c r="E247" s="2" t="inlineStr">
+        <is>
+          <t>Bremerton Marina Operations Manager</t>
+        </is>
+      </c>
+      <c r="F247" s="2" t="inlineStr">
+        <is>
+          <t>Port Of Bremerton</t>
+        </is>
+      </c>
+      <c r="G247" s="2" t="inlineStr">
+        <is>
+          <t>https://portofbremerton.org</t>
+        </is>
+      </c>
+      <c r="H247" s="2" t="inlineStr">
+        <is>
+          <t>8850 Highway 3 Southwest</t>
+        </is>
+      </c>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>Navy Yard City</t>
+        </is>
+      </c>
+      <c r="J247" s="2" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="K247" s="2" t="inlineStr">
+        <is>
+          <t>98312</t>
+        </is>
+      </c>
+      <c r="L247" s="2" t="inlineStr">
+        <is>
+          <t>Pacific Northwest - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M247" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Regulation, administration of transportation</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>Eric</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>Karacsonyi</t>
+        </is>
+      </c>
+      <c r="C248" s="2" t="inlineStr">
+        <is>
+          <t>eric@bartonandgray.com</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>2036062818</t>
+        </is>
+      </c>
+      <c r="E248" s="2" t="inlineStr">
+        <is>
+          <t>Purchasing And Supply Chain Manager</t>
+        </is>
+      </c>
+      <c r="F248" s="2" t="inlineStr">
+        <is>
+          <t>Barton &amp; Gray</t>
+        </is>
+      </c>
+      <c r="G248" s="2" t="inlineStr">
+        <is>
+          <t>https://bartonandgray.com</t>
+        </is>
+      </c>
+      <c r="H248" s="2" t="inlineStr">
+        <is>
+          <t>50 Easton Street</t>
+        </is>
+      </c>
+      <c r="I248" s="2" t="inlineStr">
+        <is>
+          <t>Nantucket</t>
+        </is>
+      </c>
+      <c r="J248" s="2" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="K248" s="2" t="inlineStr">
+        <is>
+          <t>02554</t>
+        </is>
+      </c>
+      <c r="L248" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M248" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Membership organizations, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>Rob</t>
+        </is>
+      </c>
+      <c r="B249" s="2" t="inlineStr">
+        <is>
+          <t>Wood</t>
+        </is>
+      </c>
+      <c r="C249" s="2" t="inlineStr">
+        <is>
+          <t>mrwood1@hotmail.com</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>+1 800-287-9060</t>
+        </is>
+      </c>
+      <c r="E249" s="2" t="inlineStr">
+        <is>
+          <t>Store Sales Manager</t>
+        </is>
+      </c>
+      <c r="F249" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G249" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H249" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I249" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J249" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K249" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L249" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M249" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>Greg</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>Seymour</t>
+        </is>
+      </c>
+      <c r="C250" s="2" t="inlineStr">
+        <is>
+          <t>greg@americanmarina.com</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr"/>
+      <c r="E250" s="2" t="inlineStr">
+        <is>
+          <t>General Manager Operations</t>
+        </is>
+      </c>
+      <c r="F250" s="2" t="inlineStr">
+        <is>
+          <t>American Marina</t>
+        </is>
+      </c>
+      <c r="G250" s="2" t="inlineStr">
+        <is>
+          <t>https://americanmarina.com</t>
+        </is>
+      </c>
+      <c r="H250" s="2" t="inlineStr"/>
+      <c r="I250" s="2" t="inlineStr"/>
+      <c r="J250" s="2" t="inlineStr"/>
+      <c r="K250" s="2" t="inlineStr"/>
+      <c r="L250" s="2" t="inlineStr">
+        <is>
+          <t>Other / Warm-water - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M250" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>Jacob</t>
+        </is>
+      </c>
+      <c r="B251" s="2" t="inlineStr">
+        <is>
+          <t>Dowling</t>
+        </is>
+      </c>
+      <c r="C251" s="2" t="inlineStr">
+        <is>
+          <t>jd2foot@live.com</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>+18159143594</t>
+        </is>
+      </c>
+      <c r="E251" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Store Manager</t>
+        </is>
+      </c>
+      <c r="F251" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G251" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H251" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I251" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J251" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K251" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L251" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M251" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>Alan</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>Brousseau-Works</t>
+        </is>
+      </c>
+      <c r="C252" s="2" t="inlineStr">
+        <is>
+          <t>alan@longlakemarine.com</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>+1 207-693-3159</t>
+        </is>
+      </c>
+      <c r="E252" s="2" t="inlineStr">
+        <is>
+          <t>Sales And Store Manager</t>
+        </is>
+      </c>
+      <c r="F252" s="2" t="inlineStr">
+        <is>
+          <t>Long Lake Marina, Naples Maine</t>
+        </is>
+      </c>
+      <c r="G252" s="2" t="inlineStr">
+        <is>
+          <t>https://longlakemarine.com</t>
+        </is>
+      </c>
+      <c r="H252" s="2" t="inlineStr">
+        <is>
+          <t>933 Roosevelt Trail</t>
+        </is>
+      </c>
+      <c r="I252" s="2" t="inlineStr">
+        <is>
+          <t>Naples</t>
+        </is>
+      </c>
+      <c r="J252" s="2" t="inlineStr">
+        <is>
+          <t>ME</t>
+        </is>
+      </c>
+      <c r="K252" s="2" t="inlineStr">
+        <is>
+          <t>04055</t>
+        </is>
+      </c>
+      <c r="L252" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M252" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Sporting goods and bicycle shops</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>Edward</t>
+        </is>
+      </c>
+      <c r="B253" s="2" t="inlineStr">
+        <is>
+          <t>Gillespie</t>
+        </is>
+      </c>
+      <c r="C253" s="2" t="inlineStr">
+        <is>
+          <t>egillespie@mckeegroup.net</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>+1 610-604-9800</t>
+        </is>
+      </c>
+      <c r="E253" s="2" t="inlineStr">
+        <is>
+          <t>Director  Estimating And Purchasing And Product Development</t>
+        </is>
+      </c>
+      <c r="F253" s="2" t="inlineStr">
+        <is>
+          <t>The Mckee Group</t>
+        </is>
+      </c>
+      <c r="G253" s="2" t="inlineStr">
+        <is>
+          <t>https://mckeegroup.net</t>
+        </is>
+      </c>
+      <c r="H253" s="2" t="inlineStr">
+        <is>
+          <t>940 W Sproul Rd</t>
+        </is>
+      </c>
+      <c r="I253" s="2" t="inlineStr">
+        <is>
+          <t>Springfield</t>
+        </is>
+      </c>
+      <c r="J253" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K253" s="2" t="inlineStr">
+        <is>
+          <t>19064</t>
+        </is>
+      </c>
+      <c r="L253" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M253" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Real estate agents and managers</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>Sue</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>Phelps</t>
+        </is>
+      </c>
+      <c r="C254" s="2" t="inlineStr">
+        <is>
+          <t>sphelps@lakelawnresort.com</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>2622031516</t>
+        </is>
+      </c>
+      <c r="E254" s="2" t="inlineStr">
+        <is>
+          <t>Retail Manager</t>
+        </is>
+      </c>
+      <c r="F254" s="2" t="inlineStr">
+        <is>
+          <t>Lake Lawn Resort</t>
+        </is>
+      </c>
+      <c r="G254" s="2" t="inlineStr">
+        <is>
+          <t>https://lakelawnresort.com</t>
+        </is>
+      </c>
+      <c r="H254" s="2" t="inlineStr">
+        <is>
+          <t>2400 East Geneva Street</t>
+        </is>
+      </c>
+      <c r="I254" s="2" t="inlineStr">
+        <is>
+          <t>Delavan</t>
+        </is>
+      </c>
+      <c r="J254" s="2" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="K254" s="2" t="inlineStr">
+        <is>
+          <t>53115</t>
+        </is>
+      </c>
+      <c r="L254" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M254" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Hotels and motels</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>Margaret</t>
+        </is>
+      </c>
+      <c r="B255" s="2" t="inlineStr">
+        <is>
+          <t>Timpson</t>
+        </is>
+      </c>
+      <c r="C255" s="2" t="inlineStr">
+        <is>
+          <t>megtimpson@comcast.net</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>1(717)669-6420</t>
+        </is>
+      </c>
+      <c r="E255" s="2" t="inlineStr">
+        <is>
+          <t>Sales And Merchandise Manager</t>
+        </is>
+      </c>
+      <c r="F255" s="2" t="inlineStr">
+        <is>
+          <t>New York Yacht Club</t>
+        </is>
+      </c>
+      <c r="G255" s="2" t="inlineStr">
+        <is>
+          <t>https://nyyc.org</t>
+        </is>
+      </c>
+      <c r="H255" s="2" t="inlineStr">
+        <is>
+          <t>37 West 44th Street</t>
+        </is>
+      </c>
+      <c r="I255" s="2" t="inlineStr">
+        <is>
+          <t>Ny City</t>
+        </is>
+      </c>
+      <c r="J255" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="K255" s="2" t="inlineStr">
+        <is>
+          <t>10036</t>
+        </is>
+      </c>
+      <c r="L255" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M255" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Amusement and recreation, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>Mark</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>Steffke</t>
+        </is>
+      </c>
+      <c r="C256" s="2" t="inlineStr">
+        <is>
+          <t>mark@mbyc.com</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>+13133100038</t>
+        </is>
+      </c>
+      <c r="E256" s="2" t="inlineStr">
+        <is>
+          <t>General Manager  Chief Operations Officer</t>
+        </is>
+      </c>
+      <c r="F256" s="2" t="inlineStr">
+        <is>
+          <t>Macatawa Bay Yacht Club</t>
+        </is>
+      </c>
+      <c r="G256" s="2" t="inlineStr">
+        <is>
+          <t>https://mbyc.com</t>
+        </is>
+      </c>
+      <c r="H256" s="2" t="inlineStr">
+        <is>
+          <t>2157 South Shore Drive</t>
+        </is>
+      </c>
+      <c r="I256" s="2" t="inlineStr">
+        <is>
+          <t>Macatawa</t>
+        </is>
+      </c>
+      <c r="J256" s="2" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="K256" s="2" t="inlineStr">
+        <is>
+          <t>49434</t>
+        </is>
+      </c>
+      <c r="L256" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M256" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Membership organizations, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>Rod</t>
+        </is>
+      </c>
+      <c r="B257" s="2" t="inlineStr">
+        <is>
+          <t>Bensz</t>
+        </is>
+      </c>
+      <c r="C257" s="2" t="inlineStr">
+        <is>
+          <t>rbensz@bemarine.com</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>1(219)898-3049</t>
+        </is>
+      </c>
+      <c r="E257" s="2" t="inlineStr">
+        <is>
+          <t>Director Of Sales And Owner</t>
+        </is>
+      </c>
+      <c r="F257" s="2" t="inlineStr">
+        <is>
+          <t>B&amp;E Marine</t>
+        </is>
+      </c>
+      <c r="G257" s="2" t="inlineStr">
+        <is>
+          <t>https://bemarine.com</t>
+        </is>
+      </c>
+      <c r="H257" s="2" t="inlineStr">
+        <is>
+          <t>31 Lake Shore Drive</t>
+        </is>
+      </c>
+      <c r="I257" s="2" t="inlineStr">
+        <is>
+          <t>Michiana Shrs</t>
+        </is>
+      </c>
+      <c r="J257" s="2" t="inlineStr">
+        <is>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="K257" s="2" t="inlineStr">
+        <is>
+          <t>46360</t>
+        </is>
+      </c>
+      <c r="L257" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M257" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Boat dealers</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>Streeto</t>
+        </is>
+      </c>
+      <c r="C258" s="2" t="inlineStr">
+        <is>
+          <t>antst88@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>+1 770-645-6790</t>
+        </is>
+      </c>
+      <c r="E258" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Store Manager</t>
+        </is>
+      </c>
+      <c r="F258" s="2" t="inlineStr">
+        <is>
+          <t>Pga Tour Superstore</t>
+        </is>
+      </c>
+      <c r="G258" s="2" t="inlineStr">
+        <is>
+          <t>https://pgatoursuperstore.com</t>
+        </is>
+      </c>
+      <c r="H258" s="2" t="inlineStr">
+        <is>
+          <t>1805 Old Alabama Road</t>
+        </is>
+      </c>
+      <c r="I258" s="2" t="inlineStr">
+        <is>
+          <t>Roswell</t>
+        </is>
+      </c>
+      <c r="J258" s="2" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="K258" s="2" t="inlineStr">
+        <is>
+          <t>30076</t>
+        </is>
+      </c>
+      <c r="L258" s="2" t="inlineStr">
+        <is>
+          <t>Other / Warm-water - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M258" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Sporting and recreation goods</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="B259" s="2" t="inlineStr">
+        <is>
+          <t>Brodell</t>
+        </is>
+      </c>
+      <c r="C259" s="2" t="inlineStr">
+        <is>
+          <t>brian.brodell@gmail.com</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>+1 800-287-9060</t>
+        </is>
+      </c>
+      <c r="E259" s="2" t="inlineStr">
+        <is>
+          <t>General Store Manager</t>
+        </is>
+      </c>
+      <c r="F259" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G259" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H259" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I259" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J259" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K259" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L259" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M259" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>Neal</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>Aspinall</t>
+        </is>
+      </c>
+      <c r="C260" s="2" t="inlineStr">
+        <is>
+          <t>neal@nealaspinall.com</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr"/>
+      <c r="E260" s="2" t="inlineStr">
+        <is>
+          <t>Illustrator And Graphic Designer And Owner Of The Aspinall Poster Store</t>
+        </is>
+      </c>
+      <c r="F260" s="2" t="inlineStr">
+        <is>
+          <t>Neal Aspinall Illustration &amp; Design</t>
+        </is>
+      </c>
+      <c r="G260" s="2" t="inlineStr">
+        <is>
+          <t>https://nealaspinall.com</t>
+        </is>
+      </c>
+      <c r="H260" s="2" t="inlineStr"/>
+      <c r="I260" s="2" t="inlineStr">
+        <is>
+          <t>Milwaukee</t>
+        </is>
+      </c>
+      <c r="J260" s="2" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="K260" s="2" t="inlineStr"/>
+      <c r="L260" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M260" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Commercial art and graphic design</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B261" s="2" t="inlineStr">
+        <is>
+          <t>Schaffner</t>
+        </is>
+      </c>
+      <c r="C261" s="2" t="inlineStr">
+        <is>
+          <t>dschaffner.golf@gmail.com</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>1(507)254-7436</t>
+        </is>
+      </c>
+      <c r="E261" s="2" t="inlineStr">
+        <is>
+          <t>General Sales Manager</t>
+        </is>
+      </c>
+      <c r="F261" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G261" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I261" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J261" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K261" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L261" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M261" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>Amos</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>Stephens</t>
+        </is>
+      </c>
+      <c r="C262" s="2" t="inlineStr">
+        <is>
+          <t>amosstephens@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>+1 907-376-5466</t>
+        </is>
+      </c>
+      <c r="E262" s="2" t="inlineStr">
+        <is>
+          <t>General Manager And Superintendent Of Golf Course Operations</t>
+        </is>
+      </c>
+      <c r="F262" s="2" t="inlineStr">
+        <is>
+          <t>Settlers Bay Golf Course</t>
+        </is>
+      </c>
+      <c r="G262" s="2" t="inlineStr">
+        <is>
+          <t>https://settlersbay.com</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>7307 S Frontier Dr</t>
+        </is>
+      </c>
+      <c r="I262" s="2" t="inlineStr">
+        <is>
+          <t>Meadow Lake</t>
+        </is>
+      </c>
+      <c r="J262" s="2" t="inlineStr">
+        <is>
+          <t>AK</t>
+        </is>
+      </c>
+      <c r="K262" s="2" t="inlineStr">
+        <is>
+          <t>99623</t>
+        </is>
+      </c>
+      <c r="L262" s="2" t="inlineStr">
+        <is>
+          <t>Pacific Northwest - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M262" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Membership sports and recreation clubs</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>Liz</t>
+        </is>
+      </c>
+      <c r="B263" s="2" t="inlineStr">
+        <is>
+          <t>Mernick</t>
+        </is>
+      </c>
+      <c r="C263" s="2" t="inlineStr">
+        <is>
+          <t>lmernick@libertylandingmarina.com</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>+1 201-985-8000</t>
+        </is>
+      </c>
+      <c r="E263" s="2" t="inlineStr">
+        <is>
+          <t>Store Manager</t>
+        </is>
+      </c>
+      <c r="F263" s="2" t="inlineStr">
+        <is>
+          <t>Liberty Landing Marina Llc</t>
+        </is>
+      </c>
+      <c r="G263" s="2" t="inlineStr">
+        <is>
+          <t>https://libertylandingmarina.com</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>80 Audrey Zapp Drive</t>
+        </is>
+      </c>
+      <c r="I263" s="2" t="inlineStr">
+        <is>
+          <t>Jersey City</t>
+        </is>
+      </c>
+      <c r="J263" s="2" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="K263" s="2" t="inlineStr">
+        <is>
+          <t>07305</t>
+        </is>
+      </c>
+      <c r="L263" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M263" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Prefabricated wood buildings</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>Jimmy</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>Kelsey</t>
+        </is>
+      </c>
+      <c r="C264" s="2" t="inlineStr">
+        <is>
+          <t>kelseykustoms@gmail.com</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>+1 262-275-2163</t>
+        </is>
+      </c>
+      <c r="E264" s="2" t="inlineStr">
+        <is>
+          <t>Illinois Store Manager</t>
+        </is>
+      </c>
+      <c r="F264" s="2" t="inlineStr">
+        <is>
+          <t>Gordy's Marine</t>
+        </is>
+      </c>
+      <c r="G264" s="2" t="inlineStr">
+        <is>
+          <t>https://gordysboats.com</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr">
+        <is>
+          <t>320 Lake Street</t>
+        </is>
+      </c>
+      <c r="I264" s="2" t="inlineStr">
+        <is>
+          <t>Fontana</t>
+        </is>
+      </c>
+      <c r="J264" s="2" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="K264" s="2" t="inlineStr">
+        <is>
+          <t>53125</t>
+        </is>
+      </c>
+      <c r="L264" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M264" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: New and used car dealers</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>Scott</t>
+        </is>
+      </c>
+      <c r="B265" s="2" t="inlineStr">
+        <is>
+          <t>Tucker</t>
+        </is>
+      </c>
+      <c r="C265" s="2" t="inlineStr">
+        <is>
+          <t>scott@lakespringfieldmarina.com</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>+12173411073</t>
+        </is>
+      </c>
+      <c r="E265" s="2" t="inlineStr">
+        <is>
+          <t>Salesman And Owner</t>
+        </is>
+      </c>
+      <c r="F265" s="2" t="inlineStr">
+        <is>
+          <t>Lake Springfield Marina</t>
+        </is>
+      </c>
+      <c r="G265" s="2" t="inlineStr">
+        <is>
+          <t>https://lakespringfieldmarina.com</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr">
+        <is>
+          <t>17 Waters Edge Boulevard</t>
+        </is>
+      </c>
+      <c r="I265" s="2" t="inlineStr">
+        <is>
+          <t>Springfield</t>
+        </is>
+      </c>
+      <c r="J265" s="2" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="K265" s="2" t="inlineStr">
+        <is>
+          <t>62712</t>
+        </is>
+      </c>
+      <c r="L265" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M265" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Federal reserve banks</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>Emily</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>Mero</t>
+        </is>
+      </c>
+      <c r="C266" s="2" t="inlineStr">
+        <is>
+          <t>emily@wbm.us</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>+1 518-963-7276</t>
+        </is>
+      </c>
+      <c r="E266" s="2" t="inlineStr">
+        <is>
+          <t>Assistant Store Manager</t>
+        </is>
+      </c>
+      <c r="F266" s="2" t="inlineStr">
+        <is>
+          <t>Willsboro Bay Marina, Inc</t>
+        </is>
+      </c>
+      <c r="G266" s="2" t="inlineStr">
+        <is>
+          <t>https://wbm.us</t>
+        </is>
+      </c>
+      <c r="H266" s="2" t="inlineStr">
+        <is>
+          <t>25 Klein Way</t>
+        </is>
+      </c>
+      <c r="I266" s="2" t="inlineStr">
+        <is>
+          <t>Willsboro</t>
+        </is>
+      </c>
+      <c r="J266" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="K266" s="2" t="inlineStr">
+        <is>
+          <t>12996</t>
+        </is>
+      </c>
+      <c r="L266" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M266" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Marinas</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>Ronald</t>
+        </is>
+      </c>
+      <c r="B267" s="2" t="inlineStr">
+        <is>
+          <t>Bethel</t>
+        </is>
+      </c>
+      <c r="C267" s="2" t="inlineStr">
+        <is>
+          <t>ron@certifiedsales.com</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>+1 508-478-0200</t>
+        </is>
+      </c>
+      <c r="E267" s="2" t="inlineStr">
+        <is>
+          <t>Owner  Certified Sales  Inc</t>
+        </is>
+      </c>
+      <c r="F267" s="2" t="inlineStr">
+        <is>
+          <t>Certified Sales Inc.</t>
+        </is>
+      </c>
+      <c r="G267" s="2" t="inlineStr">
+        <is>
+          <t>https://certifiedsales.com</t>
+        </is>
+      </c>
+      <c r="H267" s="2" t="inlineStr">
+        <is>
+          <t>19 Uxbridge Road</t>
+        </is>
+      </c>
+      <c r="I267" s="2" t="inlineStr">
+        <is>
+          <t>Mendon</t>
+        </is>
+      </c>
+      <c r="J267" s="2" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="K267" s="2" t="inlineStr">
+        <is>
+          <t>01756</t>
+        </is>
+      </c>
+      <c r="L267" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M267" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Business services, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>Allison</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>Johnston</t>
+        </is>
+      </c>
+      <c r="C268" s="2" t="inlineStr">
+        <is>
+          <t>lockview@aol.com</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr"/>
+      <c r="E268" s="2" t="inlineStr">
+        <is>
+          <t>Owner  Lockview Marina And Transport Co</t>
+        </is>
+      </c>
+      <c r="F268" s="2" t="inlineStr">
+        <is>
+          <t>Lockview Marina &amp; Transport</t>
+        </is>
+      </c>
+      <c r="G268" s="2" t="inlineStr"/>
+      <c r="H268" s="2" t="inlineStr"/>
+      <c r="I268" s="2" t="inlineStr"/>
+      <c r="J268" s="2" t="inlineStr"/>
+      <c r="K268" s="2" t="inlineStr"/>
+      <c r="L268" s="2" t="inlineStr">
+        <is>
+          <t>Other / Warm-water - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M268" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>Terry</t>
+        </is>
+      </c>
+      <c r="B269" s="2" t="inlineStr">
+        <is>
+          <t>Risteen</t>
+        </is>
+      </c>
+      <c r="C269" s="2" t="inlineStr">
+        <is>
+          <t>taristeen@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>+1 508-233-4172</t>
+        </is>
+      </c>
+      <c r="E269" s="2" t="inlineStr">
+        <is>
+          <t>Store Divisional Manager</t>
+        </is>
+      </c>
+      <c r="F269" s="2" t="inlineStr">
+        <is>
+          <t>Navy Exchange Service Command (Nexcom)</t>
+        </is>
+      </c>
+      <c r="G269" s="2" t="inlineStr">
+        <is>
+          <t>https://navyexchange.jobs</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t>Natick Army Base</t>
+        </is>
+      </c>
+      <c r="I269" s="2" t="inlineStr">
+        <is>
+          <t>Natick</t>
+        </is>
+      </c>
+      <c r="J269" s="2" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="K269" s="2" t="inlineStr">
+        <is>
+          <t>01760</t>
+        </is>
+      </c>
+      <c r="L269" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M269" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Variety stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>Mike</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>Thuemmler</t>
+        </is>
+      </c>
+      <c r="C270" s="2" t="inlineStr">
+        <is>
+          <t>dockmaster@sanduskyyachtclub.com</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>+1 419-625-6567</t>
+        </is>
+      </c>
+      <c r="E270" s="2" t="inlineStr">
+        <is>
+          <t>General Manager And Chief Operations Officer</t>
+        </is>
+      </c>
+      <c r="F270" s="2" t="inlineStr">
+        <is>
+          <t>Sandusky Yacht Club</t>
+        </is>
+      </c>
+      <c r="G270" s="2" t="inlineStr">
+        <is>
+          <t>https://sanduskyyachtclub.com</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>529 East Water Street</t>
+        </is>
+      </c>
+      <c r="I270" s="2" t="inlineStr">
+        <is>
+          <t>Pt Clinton</t>
+        </is>
+      </c>
+      <c r="J270" s="2" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="K270" s="2" t="inlineStr">
+        <is>
+          <t>43452</t>
+        </is>
+      </c>
+      <c r="L270" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M270" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Communication services, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="B271" s="2" t="inlineStr">
+        <is>
+          <t>Vasil</t>
+        </is>
+      </c>
+      <c r="C271" s="2" t="inlineStr">
+        <is>
+          <t>danvasil31@gmail.com</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>1(848)525-7800</t>
+        </is>
+      </c>
+      <c r="E271" s="2" t="inlineStr">
+        <is>
+          <t>General Sales Manager</t>
+        </is>
+      </c>
+      <c r="F271" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G271" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H271" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I271" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J271" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K271" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L271" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M271" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>Toledo</t>
+        </is>
+      </c>
+      <c r="C272" s="2" t="inlineStr">
+        <is>
+          <t>dtoledo@jordache.com</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>+1 212-944-1330</t>
+        </is>
+      </c>
+      <c r="E272" s="2" t="inlineStr">
+        <is>
+          <t>Sourcing And Production Manager</t>
+        </is>
+      </c>
+      <c r="F272" s="2" t="inlineStr">
+        <is>
+          <t>Jordache</t>
+        </is>
+      </c>
+      <c r="G272" s="2" t="inlineStr">
+        <is>
+          <t>https://jordache.com</t>
+        </is>
+      </c>
+      <c r="H272" s="2" t="inlineStr">
+        <is>
+          <t>1400 Broadway</t>
+        </is>
+      </c>
+      <c r="I272" s="2" t="inlineStr">
+        <is>
+          <t>Nyc</t>
+        </is>
+      </c>
+      <c r="J272" s="2" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="K272" s="2" t="inlineStr">
+        <is>
+          <t>10018</t>
+        </is>
+      </c>
+      <c r="L272" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M272" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Men's and boys' clothing stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>Molly</t>
+        </is>
+      </c>
+      <c r="B273" s="2" t="inlineStr">
+        <is>
+          <t>Miller</t>
+        </is>
+      </c>
+      <c r="C273" s="2" t="inlineStr">
+        <is>
+          <t>m.miller@pittrace.com</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>+1 724-535-1000</t>
+        </is>
+      </c>
+      <c r="E273" s="2" t="inlineStr">
+        <is>
+          <t>Retail Sales Manager</t>
+        </is>
+      </c>
+      <c r="F273" s="2" t="inlineStr">
+        <is>
+          <t>Pittsburgh International Race Complex</t>
+        </is>
+      </c>
+      <c r="G273" s="2" t="inlineStr">
+        <is>
+          <t>https://pittrace.com</t>
+        </is>
+      </c>
+      <c r="H273" s="2" t="inlineStr">
+        <is>
+          <t>201 Penndale Road</t>
+        </is>
+      </c>
+      <c r="I273" s="2" t="inlineStr">
+        <is>
+          <t>Wampum</t>
+        </is>
+      </c>
+      <c r="J273" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K273" s="2" t="inlineStr">
+        <is>
+          <t>16157</t>
+        </is>
+      </c>
+      <c r="L273" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M273" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Sports clubs, managers, and promoters</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>Karen</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>Shea</t>
+        </is>
+      </c>
+      <c r="C274" s="2" t="inlineStr">
+        <is>
+          <t>newport@nicholsonyachts.com</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>+1 401-849-0344</t>
+        </is>
+      </c>
+      <c r="E274" s="2" t="inlineStr">
+        <is>
+          <t>Owner And Yacht Charters And Yacht Sales And Nicholson Yachts Worldwide</t>
+        </is>
+      </c>
+      <c r="F274" s="2" t="inlineStr">
+        <is>
+          <t>Nicholson Yachts Worldwide</t>
+        </is>
+      </c>
+      <c r="G274" s="2" t="inlineStr">
+        <is>
+          <t>https://nicholsonyachts.com</t>
+        </is>
+      </c>
+      <c r="H274" s="2" t="inlineStr">
+        <is>
+          <t>1 Washington Street</t>
+        </is>
+      </c>
+      <c r="I274" s="2" t="inlineStr">
+        <is>
+          <t>Newport</t>
+        </is>
+      </c>
+      <c r="J274" s="2" t="inlineStr">
+        <is>
+          <t>RI</t>
+        </is>
+      </c>
+      <c r="K274" s="2" t="inlineStr">
+        <is>
+          <t>02840</t>
+        </is>
+      </c>
+      <c r="L274" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M274" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Amusement and recreation, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>Holly</t>
+        </is>
+      </c>
+      <c r="B275" s="2" t="inlineStr">
+        <is>
+          <t>Mcgory</t>
+        </is>
+      </c>
+      <c r="C275" s="2" t="inlineStr">
+        <is>
+          <t>hmcgory@aol.com</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>+1 419-433-3800</t>
+        </is>
+      </c>
+      <c r="E275" s="2" t="inlineStr">
+        <is>
+          <t>General Merchandise Manager</t>
+        </is>
+      </c>
+      <c r="F275" s="2" t="inlineStr">
+        <is>
+          <t>Sawmill Creek Resort</t>
+        </is>
+      </c>
+      <c r="G275" s="2" t="inlineStr">
+        <is>
+          <t>https://sawmillcreekresort.com</t>
+        </is>
+      </c>
+      <c r="H275" s="2" t="inlineStr">
+        <is>
+          <t>400 Sawmill Creek Drive West</t>
+        </is>
+      </c>
+      <c r="I275" s="2" t="inlineStr">
+        <is>
+          <t>Ruggles Beach</t>
+        </is>
+      </c>
+      <c r="J275" s="2" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="K275" s="2" t="inlineStr">
+        <is>
+          <t>44839</t>
+        </is>
+      </c>
+      <c r="L275" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M275" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Hotels and motels</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>Price</t>
+        </is>
+      </c>
+      <c r="C276" s="2" t="inlineStr">
+        <is>
+          <t>price434@msn.com</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>+17346648300</t>
+        </is>
+      </c>
+      <c r="E276" s="2" t="inlineStr">
+        <is>
+          <t>General Manager Chief Operations Officer</t>
+        </is>
+      </c>
+      <c r="F276" s="2" t="inlineStr">
+        <is>
+          <t>Detroit Yacht Club</t>
+        </is>
+      </c>
+      <c r="G276" s="2" t="inlineStr">
+        <is>
+          <t>https://dyc.com</t>
+        </is>
+      </c>
+      <c r="H276" s="2" t="inlineStr">
+        <is>
+          <t>1 Riverbank Road</t>
+        </is>
+      </c>
+      <c r="I276" s="2" t="inlineStr">
+        <is>
+          <t>Detroit</t>
+        </is>
+      </c>
+      <c r="J276" s="2" t="inlineStr">
+        <is>
+          <t>MI</t>
+        </is>
+      </c>
+      <c r="K276" s="2" t="inlineStr">
+        <is>
+          <t>48207</t>
+        </is>
+      </c>
+      <c r="L276" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M276" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Amusement and recreation, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>Ivan</t>
+        </is>
+      </c>
+      <c r="B277" s="2" t="inlineStr">
+        <is>
+          <t>Garcia</t>
+        </is>
+      </c>
+      <c r="C277" s="2" t="inlineStr">
+        <is>
+          <t>caprichos@gmail.com</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>+19737894645</t>
+        </is>
+      </c>
+      <c r="E277" s="2" t="inlineStr">
+        <is>
+          <t>Store Manager</t>
+        </is>
+      </c>
+      <c r="F277" s="2" t="inlineStr">
+        <is>
+          <t>Liberty Landing Marina Llc</t>
+        </is>
+      </c>
+      <c r="G277" s="2" t="inlineStr">
+        <is>
+          <t>https://libertylandingmarina.com</t>
+        </is>
+      </c>
+      <c r="H277" s="2" t="inlineStr">
+        <is>
+          <t>80 Audrey Zapp Drive</t>
+        </is>
+      </c>
+      <c r="I277" s="2" t="inlineStr">
+        <is>
+          <t>Jersey City</t>
+        </is>
+      </c>
+      <c r="J277" s="2" t="inlineStr">
+        <is>
+          <t>NJ</t>
+        </is>
+      </c>
+      <c r="K277" s="2" t="inlineStr">
+        <is>
+          <t>07305</t>
+        </is>
+      </c>
+      <c r="L277" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M277" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Prefabricated wood buildings</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>Deb</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>Stockman</t>
+        </is>
+      </c>
+      <c r="C278" s="2" t="inlineStr">
+        <is>
+          <t>dandr8256@msn.com</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>+1 508-233-4172</t>
+        </is>
+      </c>
+      <c r="E278" s="2" t="inlineStr">
+        <is>
+          <t>Merchandise Manager</t>
+        </is>
+      </c>
+      <c r="F278" s="2" t="inlineStr">
+        <is>
+          <t>Navy Exchange Service Command (Nexcom)</t>
+        </is>
+      </c>
+      <c r="G278" s="2" t="inlineStr">
+        <is>
+          <t>https://navyexchange.jobs</t>
+        </is>
+      </c>
+      <c r="H278" s="2" t="inlineStr">
+        <is>
+          <t>Natick Army Base</t>
+        </is>
+      </c>
+      <c r="I278" s="2" t="inlineStr">
+        <is>
+          <t>Natick</t>
+        </is>
+      </c>
+      <c r="J278" s="2" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="K278" s="2" t="inlineStr">
+        <is>
+          <t>01760</t>
+        </is>
+      </c>
+      <c r="L278" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M278" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Variety stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>Kenneth</t>
+        </is>
+      </c>
+      <c r="B279" s="2" t="inlineStr">
+        <is>
+          <t>York</t>
+        </is>
+      </c>
+      <c r="C279" s="2" t="inlineStr">
+        <is>
+          <t>ahsbballa30@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>+13176250448</t>
+        </is>
+      </c>
+      <c r="E279" s="2" t="inlineStr">
+        <is>
+          <t>General Sales Manager</t>
+        </is>
+      </c>
+      <c r="F279" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G279" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H279" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I279" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J279" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K279" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L279" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M279" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>Matt</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>Michael</t>
+        </is>
+      </c>
+      <c r="C280" s="2" t="inlineStr">
+        <is>
+          <t>mattmich@comcast.net</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>+1 414-271-4455</t>
+        </is>
+      </c>
+      <c r="E280" s="2" t="inlineStr">
+        <is>
+          <t>General Manager And Chief Operations Officer</t>
+        </is>
+      </c>
+      <c r="F280" s="2" t="inlineStr">
+        <is>
+          <t>Milwaukee Yacht Club</t>
+        </is>
+      </c>
+      <c r="G280" s="2" t="inlineStr">
+        <is>
+          <t>https://milwaukeeyc.com</t>
+        </is>
+      </c>
+      <c r="H280" s="2" t="inlineStr">
+        <is>
+          <t>1700 N Lincoln Memorial Dr</t>
+        </is>
+      </c>
+      <c r="I280" s="2" t="inlineStr">
+        <is>
+          <t>Milwaukee</t>
+        </is>
+      </c>
+      <c r="J280" s="2" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="K280" s="2" t="inlineStr">
+        <is>
+          <t>53202</t>
+        </is>
+      </c>
+      <c r="L280" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M280" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Sports clubs, managers, and promoters</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>Vicki</t>
+        </is>
+      </c>
+      <c r="B281" s="2" t="inlineStr">
+        <is>
+          <t>Main</t>
+        </is>
+      </c>
+      <c r="C281" s="2" t="inlineStr">
+        <is>
+          <t>vmain@eagleridge.com</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>+1 815-777-5000</t>
+        </is>
+      </c>
+      <c r="E281" s="2" t="inlineStr">
+        <is>
+          <t>Merchandise Manager</t>
+        </is>
+      </c>
+      <c r="F281" s="2" t="inlineStr">
+        <is>
+          <t>Eagle Ridge Resort &amp; Spa</t>
+        </is>
+      </c>
+      <c r="G281" s="2" t="inlineStr">
+        <is>
+          <t>https://eagleridge.com</t>
+        </is>
+      </c>
+      <c r="H281" s="2" t="inlineStr">
+        <is>
+          <t>444 Eagle Ridge Drive</t>
+        </is>
+      </c>
+      <c r="I281" s="2" t="inlineStr">
+        <is>
+          <t>Galena</t>
+        </is>
+      </c>
+      <c r="J281" s="2" t="inlineStr">
+        <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="K281" s="2" t="inlineStr">
+        <is>
+          <t>61036</t>
+        </is>
+      </c>
+      <c r="L281" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M281" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Hotels and motels</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>Paula</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>Fronk</t>
+        </is>
+      </c>
+      <c r="C282" s="2" t="inlineStr">
+        <is>
+          <t>mercgirl1975@gmail.com</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr"/>
+      <c r="E282" s="2" t="inlineStr">
+        <is>
+          <t>General Manager Sales And Finacial</t>
+        </is>
+      </c>
+      <c r="F282" s="2" t="inlineStr">
+        <is>
+          <t>Lake Holcombe Marina</t>
+        </is>
+      </c>
+      <c r="G282" s="2" t="inlineStr">
+        <is>
+          <t>https://lakeholcombemarina.com</t>
+        </is>
+      </c>
+      <c r="H282" s="2" t="inlineStr"/>
+      <c r="I282" s="2" t="inlineStr"/>
+      <c r="J282" s="2" t="inlineStr"/>
+      <c r="K282" s="2" t="inlineStr"/>
+      <c r="L282" s="2" t="inlineStr">
+        <is>
+          <t>Other / Warm-water - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M282" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>Pat</t>
+        </is>
+      </c>
+      <c r="B283" s="2" t="inlineStr">
+        <is>
+          <t>Marek</t>
+        </is>
+      </c>
+      <c r="C283" s="2" t="inlineStr">
+        <is>
+          <t>pmarek1328@msn.com</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>+1 800-287-9060</t>
+        </is>
+      </c>
+      <c r="E283" s="2" t="inlineStr">
+        <is>
+          <t>Store Manager</t>
+        </is>
+      </c>
+      <c r="F283" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G283" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H283" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I283" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J283" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K283" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L283" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M283" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>Stephen</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>Creese</t>
+        </is>
+      </c>
+      <c r="C284" s="2" t="inlineStr">
+        <is>
+          <t>screese@ghyc.com</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>+15082213409</t>
+        </is>
+      </c>
+      <c r="E284" s="2" t="inlineStr">
+        <is>
+          <t>General Manager And Chief Operations Officer</t>
+        </is>
+      </c>
+      <c r="F284" s="2" t="inlineStr">
+        <is>
+          <t>Great Harbor Yacht Club</t>
+        </is>
+      </c>
+      <c r="G284" s="2" t="inlineStr">
+        <is>
+          <t>https://ghyc.com</t>
+        </is>
+      </c>
+      <c r="H284" s="2" t="inlineStr">
+        <is>
+          <t>23 Nobadeer Farm Rd</t>
+        </is>
+      </c>
+      <c r="I284" s="2" t="inlineStr">
+        <is>
+          <t>Nantucket</t>
+        </is>
+      </c>
+      <c r="J284" s="2" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="K284" s="2" t="inlineStr">
+        <is>
+          <t>02554</t>
+        </is>
+      </c>
+      <c r="L284" s="2" t="inlineStr">
+        <is>
+          <t>Northeast - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M284" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Beauty shops</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>Daniel</t>
+        </is>
+      </c>
+      <c r="B285" s="2" t="inlineStr">
+        <is>
+          <t>Tomasetti</t>
+        </is>
+      </c>
+      <c r="C285" s="2" t="inlineStr">
+        <is>
+          <t>danieltomasetti@hotmail.com</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>54 11 4000 4500</t>
+        </is>
+      </c>
+      <c r="E285" s="2" t="inlineStr">
+        <is>
+          <t>Spare Parts Purchase   Chief</t>
+        </is>
+      </c>
+      <c r="F285" s="2" t="inlineStr">
+        <is>
+          <t>Honda Motor De Argentina</t>
+        </is>
+      </c>
+      <c r="G285" s="2" t="inlineStr">
+        <is>
+          <t>https://honda.com.ar</t>
+        </is>
+      </c>
+      <c r="H285" s="2" t="inlineStr">
+        <is>
+          <t>2-1-1, Minamiaoyama</t>
+        </is>
+      </c>
+      <c r="I285" s="2" t="inlineStr">
+        <is>
+          <t>Minato-Ku</t>
+        </is>
+      </c>
+      <c r="J285" s="2" t="inlineStr"/>
+      <c r="K285" s="2" t="inlineStr">
+        <is>
+          <t>107-0062</t>
+        </is>
+      </c>
+      <c r="L285" s="2" t="inlineStr">
+        <is>
+          <t>Other / Warm-water - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M285" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Motor vehicles and car bodies</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>Tom</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>Martin</t>
+        </is>
+      </c>
+      <c r="C286" s="2" t="inlineStr">
+        <is>
+          <t>tmarty0225@gmail.com</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>+17087382024</t>
+        </is>
+      </c>
+      <c r="E286" s="2" t="inlineStr">
+        <is>
+          <t>General Sales Manager</t>
+        </is>
+      </c>
+      <c r="F286" s="2" t="inlineStr">
+        <is>
+          <t>Golf Galaxy</t>
+        </is>
+      </c>
+      <c r="G286" s="2" t="inlineStr">
+        <is>
+          <t>https://golfgalaxy.com</t>
+        </is>
+      </c>
+      <c r="H286" s="2" t="inlineStr">
+        <is>
+          <t>345 Court Street</t>
+        </is>
+      </c>
+      <c r="I286" s="2" t="inlineStr">
+        <is>
+          <t>Coropolis</t>
+        </is>
+      </c>
+      <c r="J286" s="2" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="K286" s="2" t="inlineStr">
+        <is>
+          <t>15108</t>
+        </is>
+      </c>
+      <c r="L286" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M286" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Jewelry stores</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="B287" s="2" t="inlineStr">
+        <is>
+          <t>Drapeau</t>
+        </is>
+      </c>
+      <c r="C287" s="2" t="inlineStr">
+        <is>
+          <t>dickdrapo@yahoo.com</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>+65 6887 4335</t>
+        </is>
+      </c>
+      <c r="E287" s="2" t="inlineStr">
+        <is>
+          <t>Owner Representative For Construction</t>
+        </is>
+      </c>
+      <c r="F287" s="2" t="inlineStr">
+        <is>
+          <t>Self Leadership International ★ Leadership Development</t>
+        </is>
+      </c>
+      <c r="G287" s="2" t="inlineStr">
+        <is>
+          <t>https://selfleadership.com</t>
+        </is>
+      </c>
+      <c r="H287" s="2" t="inlineStr">
+        <is>
+          <t>1 Raffles Place</t>
+        </is>
+      </c>
+      <c r="I287" s="2" t="inlineStr">
+        <is>
+          <t>Singapore</t>
+        </is>
+      </c>
+      <c r="J287" s="2" t="inlineStr"/>
+      <c r="K287" s="2" t="inlineStr"/>
+      <c r="L287" s="2" t="inlineStr">
+        <is>
+          <t>Other / Warm-water - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M287" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Vocational schools, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>David</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>Dunn</t>
+        </is>
+      </c>
+      <c r="C288" s="2" t="inlineStr">
+        <is>
+          <t>ddunn@sanduskyyachtclub.com</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>1(989)996-0064</t>
+        </is>
+      </c>
+      <c r="E288" s="2" t="inlineStr">
+        <is>
+          <t>General Manager And Chief Operations Officer</t>
+        </is>
+      </c>
+      <c r="F288" s="2" t="inlineStr">
+        <is>
+          <t>Sandusky Yacht Club</t>
+        </is>
+      </c>
+      <c r="G288" s="2" t="inlineStr">
+        <is>
+          <t>https://sanduskyyachtclub.com</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="inlineStr">
+        <is>
+          <t>529 East Water Street</t>
+        </is>
+      </c>
+      <c r="I288" s="2" t="inlineStr">
+        <is>
+          <t>Pt Clinton</t>
+        </is>
+      </c>
+      <c r="J288" s="2" t="inlineStr">
+        <is>
+          <t>OH</t>
+        </is>
+      </c>
+      <c r="K288" s="2" t="inlineStr">
+        <is>
+          <t>43452</t>
+        </is>
+      </c>
+      <c r="L288" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M288" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Communication services, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>Tim</t>
+        </is>
+      </c>
+      <c r="B289" s="2" t="inlineStr">
+        <is>
+          <t>Hummel</t>
+        </is>
+      </c>
+      <c r="C289" s="2" t="inlineStr">
+        <is>
+          <t>tacomayachtclub@aol.com</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>+1 941-365-4191</t>
+        </is>
+      </c>
+      <c r="E289" s="2" t="inlineStr">
+        <is>
+          <t>Chief Operations Officer And General Manager</t>
+        </is>
+      </c>
+      <c r="F289" s="2" t="inlineStr">
+        <is>
+          <t>Tacoma Yacht Club</t>
+        </is>
+      </c>
+      <c r="G289" s="2" t="inlineStr">
+        <is>
+          <t>https://tacomayachtclub.org</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t>3502 N Union Ave</t>
+        </is>
+      </c>
+      <c r="I289" s="2" t="inlineStr">
+        <is>
+          <t>Ruston</t>
+        </is>
+      </c>
+      <c r="J289" s="2" t="inlineStr">
+        <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="K289" s="2" t="inlineStr">
+        <is>
+          <t>98407</t>
+        </is>
+      </c>
+      <c r="L289" s="2" t="inlineStr">
+        <is>
+          <t>Pacific Northwest - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M289" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Business services, nec</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>Sean</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>Keith</t>
+        </is>
+      </c>
+      <c r="C290" s="2" t="inlineStr">
+        <is>
+          <t>keith@keithsmarina.com</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>+1 262-334-9389</t>
+        </is>
+      </c>
+      <c r="E290" s="2" t="inlineStr">
+        <is>
+          <t>Owner And Sales</t>
+        </is>
+      </c>
+      <c r="F290" s="2" t="inlineStr">
+        <is>
+          <t>Keith's Marina</t>
+        </is>
+      </c>
+      <c r="G290" s="2" t="inlineStr">
+        <is>
+          <t>https://keithsmarina.com</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t>4339 Wi 33</t>
+        </is>
+      </c>
+      <c r="I290" s="2" t="inlineStr">
+        <is>
+          <t>West Bend</t>
+        </is>
+      </c>
+      <c r="J290" s="2" t="inlineStr">
+        <is>
+          <t>WI</t>
+        </is>
+      </c>
+      <c r="K290" s="2" t="inlineStr">
+        <is>
+          <t>53095</t>
+        </is>
+      </c>
+      <c r="L290" s="2" t="inlineStr">
+        <is>
+          <t>Great Lakes - BookYourData import</t>
+        </is>
+      </c>
+      <c r="M290" s="2" t="inlineStr">
+        <is>
+          <t>Source: BookYourData list; email status: Deliverable; industry: Boat dealers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M241"/>
+  <autoFilter ref="A1:M290"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>